<commit_message>
GRC Risk Register - with control testing
</commit_message>
<xml_diff>
--- a/Amazon Supply Chain GRC Risk Register.xlsx
+++ b/Amazon Supply Chain GRC Risk Register.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk_Register" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control_Testing_Log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,8 +51,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -94,8 +103,28 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2D3D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -205,11 +234,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -256,6 +299,22 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1078,8 +1137,16 @@
       </c>
       <c r="P4" s="6" t="n"/>
       <c r="Q4" s="6" t="n"/>
-      <c r="R4" s="6" t="n"/>
-      <c r="S4" s="6" t="n"/>
+      <c r="R4" s="18" t="inlineStr">
+        <is>
+          <t>Control Tests</t>
+        </is>
+      </c>
+      <c r="S4" s="18" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="23.5" customHeight="1">
       <c r="A5" s="6" t="n"/>
@@ -1122,8 +1189,15 @@
       </c>
       <c r="P5" s="6" t="n"/>
       <c r="Q5" s="6" t="n"/>
-      <c r="R5" s="6" t="n"/>
-      <c r="S5" s="6" t="n"/>
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>Total Tests</t>
+        </is>
+      </c>
+      <c r="S5" s="6">
+        <f>COUNTA(Control_Testing_Log!A2:A100)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
@@ -1157,8 +1231,15 @@
       </c>
       <c r="P6" s="6" t="n"/>
       <c r="Q6" s="6" t="n"/>
-      <c r="R6" s="6" t="n"/>
-      <c r="S6" s="6" t="n"/>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>Effective</t>
+        </is>
+      </c>
+      <c r="S6" s="6">
+        <f>COUNTIF(Control_Testing_Log!K:K, "Effective")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
@@ -1192,8 +1273,15 @@
       </c>
       <c r="P7" s="6" t="n"/>
       <c r="Q7" s="6" t="n"/>
-      <c r="R7" s="6" t="n"/>
-      <c r="S7" s="6" t="n"/>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>Partially Effective / Exception</t>
+        </is>
+      </c>
+      <c r="S7" s="6">
+        <f>COUNTIF(Control_Testing_Log!K:K, "*Effective*")-COUNTIF(Control_Testing_Log!K:K, "Effective")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
@@ -1227,8 +1315,15 @@
       </c>
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="6" t="n"/>
-      <c r="R8" s="6" t="n"/>
-      <c r="S8" s="6" t="n"/>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>Ineffective</t>
+        </is>
+      </c>
+      <c r="S8" s="6">
+        <f>COUNTIF(Control_Testing_Log!K:K, "Ineffective")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -6702,4 +6797,466 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="19" t="inlineStr">
+        <is>
+          <t>Related Risk ID(s)</t>
+        </is>
+      </c>
+      <c r="C1" s="19" t="inlineStr">
+        <is>
+          <t>Control Name</t>
+        </is>
+      </c>
+      <c r="D1" s="19" t="inlineStr">
+        <is>
+          <t>Control Owner</t>
+        </is>
+      </c>
+      <c r="E1" s="19" t="inlineStr">
+        <is>
+          <t>NIST CSF Function</t>
+        </is>
+      </c>
+      <c r="F1" s="19" t="inlineStr">
+        <is>
+          <t>Test Objective</t>
+        </is>
+      </c>
+      <c r="G1" s="19" t="inlineStr">
+        <is>
+          <t>Test Procedure Performed</t>
+        </is>
+      </c>
+      <c r="H1" s="19" t="inlineStr">
+        <is>
+          <t>Evidence Reviewed</t>
+        </is>
+      </c>
+      <c r="I1" s="19" t="inlineStr">
+        <is>
+          <t>Sample Size</t>
+        </is>
+      </c>
+      <c r="J1" s="19" t="inlineStr">
+        <is>
+          <t>Test Date</t>
+        </is>
+      </c>
+      <c r="K1" s="19" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="L1" s="19" t="inlineStr">
+        <is>
+          <t>Finding / Exception</t>
+        </is>
+      </c>
+      <c r="M1" s="19" t="inlineStr">
+        <is>
+          <t>Recommended Remediation</t>
+        </is>
+      </c>
+      <c r="N1" s="19" t="inlineStr">
+        <is>
+          <t>Tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>CT-001</t>
+        </is>
+      </c>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>R-008, R-011, R-022, R-029, R-034, R-038, R-044, R-050</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>Annual Access Reviews (Cloud Admin Privileged Access)</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>Cloud Sec</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>Identify / Protect</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>Verify privileged cloud admin access is reviewed at least annually and access no longer required is revoked timely.</t>
+        </is>
+      </c>
+      <c r="G2" s="20" t="inlineStr">
+        <is>
+          <t>Selected a sample of 15 privileged cloud admin accounts across NA, EU, APAC, and LATAM from the most recent access-review cycle. Confirmed each had a documented sign-off within 12 months, and traced 5 'access revoked' decisions to confirm actual deprovisioning within 5 business days.</t>
+        </is>
+      </c>
+      <c r="H2" s="20" t="inlineStr">
+        <is>
+          <t>Access review sign-off log (Q2 2026), IAM deprovisioning audit trail, sample account list.</t>
+        </is>
+      </c>
+      <c r="I2" s="20" t="inlineStr">
+        <is>
+          <t>15 of ~140 privileged accounts</t>
+        </is>
+      </c>
+      <c r="J2" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K2" s="21" t="inlineStr">
+        <is>
+          <t>Partially Effective</t>
+        </is>
+      </c>
+      <c r="L2" s="20" t="inlineStr">
+        <is>
+          <t>3 of 15 sampled accounts (20%) had review sign-offs completed but access was not revoked in the IAM system for 12-19 days after the 'revoke' decision, exceeding the 5-business-day SLA. Root cause: manual deprovisioning process with no system-enforced deadline.</t>
+        </is>
+      </c>
+      <c r="M2" s="20" t="inlineStr">
+        <is>
+          <t>Implement automated deprovisioning triggered directly by access-review decisions rather than a manual follow-up ticket.</t>
+        </is>
+      </c>
+      <c r="N2" s="20" t="inlineStr">
+        <is>
+          <t>A. Rehman</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>CT-002</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>R-014, R-037, R-041, R-043, R-045, R-048, R-049</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Warehouse IoT Network Segmentation</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>OT Security</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>Protect / Detect</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>Verify warehouse IoT devices (barcode scanners, sortation sensors) are logically segmented from the corporate network.</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Reviewed network architecture diagrams for 3 warehouse sites (NA, EU, APAC). Reviewed firewall/VLAN configuration exports confirming IoT VLAN isolation, and checked for exception/bridge rules allowing IoT-to-corporate traffic.</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>Network architecture diagrams, firewall rule exports, VLAN configuration records.</t>
+        </is>
+      </c>
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>3 of 22 warehouse sites</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K3" s="21" t="inlineStr">
+        <is>
+          <t>Effective (1 exception)</t>
+        </is>
+      </c>
+      <c r="L3" s="20" t="inlineStr">
+        <is>
+          <t>2 of 3 sites had clean segmentation with no cross-VLAN exceptions. 1 site (APAC) had a temporary firewall rule opened for a vendor maintenance visit 4 months prior that was never closed, allowing IoT VLAN traffic to reach a corporate file share.</t>
+        </is>
+      </c>
+      <c r="M3" s="20" t="inlineStr">
+        <is>
+          <t>Implement a firewall exception expiration/auto-review process for all vendor-maintenance-related temporary rules.</t>
+        </is>
+      </c>
+      <c r="N3" s="20" t="inlineStr">
+        <is>
+          <t>A. Rehman</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>CT-003</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>R-018, R-023, R-030, R-032</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>HR Portal Authentication Controls</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Identity Team</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Protect</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>Determine whether password complexity rules are sufficient to mitigate unauthorized access in the continued absence of MFA.</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Reviewed HR portal authentication configuration and password policy settings. Checked whether elevated-access HR admin accounts had MFA enforced despite the general population not having it. Reviewed 90 days of failed-login/lockout logs for credential-stuffing indicators.</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="inlineStr">
+        <is>
+          <t>Authentication configuration export, password policy documentation, 90-day failed-login log.</t>
+        </is>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>Full population, 90-day window</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="K4" s="22" t="inlineStr">
+        <is>
+          <t>Ineffective</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="inlineStr">
+        <is>
+          <t>Password complexity alone does not constitute an adequate compensating control for the absence of MFA on a system handling PII (per NIST 800-63B). Failed-login logs showed 340 failed attempts across 22 accounts in 90 days, consistent with credential-stuffing patterns, with no automated lockout until the 10th consecutive failure.</t>
+        </is>
+      </c>
+      <c r="M4" s="20" t="inlineStr">
+        <is>
+          <t>Prioritize MFA enforcement on the HR portal as a Critical remediation item (tracked as R-018/023/030/032); reduce lockout threshold to 5 attempts in the interim.</t>
+        </is>
+      </c>
+      <c r="N4" s="20" t="inlineStr">
+        <is>
+          <t>A. Rehman</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>CT-004</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>R-015, R-020, R-021, R-042</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>Third-Party Vendor Remote Access (VPN)</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Vendor Risk</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Protect</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>Verify third-party HVAC/facilities vendors are restricted to least-privilege VPN access and deprovisioned when contracts end.</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>Selected a sample of 8 active third-party vendor VPN accounts. Confirmed each was tied to an active, unexpired vendor contract, and verified VPN access scope was restricted to building-management-system IP ranges only.</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>Vendor contract register, VPN access-grant list, network access-scope configuration.</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>8 of 19 active third-party VPN accounts</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="K5" s="23" t="inlineStr">
+        <is>
+          <t>Effective</t>
+        </is>
+      </c>
+      <c r="L5" s="20" t="inlineStr">
+        <is>
+          <t>All 8 sampled accounts were correctly scoped and tied to active contracts. No exceptions noted.</t>
+        </is>
+      </c>
+      <c r="M5" s="20" t="inlineStr">
+        <is>
+          <t>None required; expand sample size in the next testing cycle given population size.</t>
+        </is>
+      </c>
+      <c r="N5" s="20" t="inlineStr">
+        <is>
+          <t>A. Rehman</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>CT-005</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>R-019, R-024, R-033</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Regional Backup &amp; Recovery Testing</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>Disaster Recovery</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>Recover</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>Verify weekly cloud backups for APAC regional systems can be successfully restored within the recovery time objective (RTO).</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Confirmed backup job completion logs for the last 8 weekly cycles. Requested evidence of the most recent backup restoration test for the APAC region.</t>
+        </is>
+      </c>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>Backup job completion logs (8-week window), disaster recovery test records.</t>
+        </is>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>8 of 8 backup cycles; 1 restoration test record requested</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="inlineStr">
+        <is>
+          <t>Ineffective</t>
+        </is>
+      </c>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>All 8 weekly backup jobs completed successfully, but no backup restoration test has been performed for the APAC region in over 18 months. Backup existence was confirmed; recoverability was not.</t>
+        </is>
+      </c>
+      <c r="M6" s="20" t="inlineStr">
+        <is>
+          <t>Schedule and execute a full restoration test for the APAC region within 30 days; establish a semi-annual restoration-testing cadence for all regions.</t>
+        </is>
+      </c>
+      <c r="N6" s="20" t="inlineStr">
+        <is>
+          <t>A. Rehman</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>